<commit_message>
deploy: feature/careteam → branches/feature-careteam a0d1bbde8827a1ac958e87d20b4840ac465ed05c
</commit_message>
<xml_diff>
--- a/branches/feature-careteam/StructureDefinition-riv-care-manager-careteam.xlsx
+++ b/branches/feature-careteam/StructureDefinition-riv-care-manager-careteam.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-15T12:03:42+00:00</t>
+    <t>2026-10-15T12:49:20+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1002,7 +1002,7 @@
   </si>
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-fast-kontakt-typ-kod-eller-text:Typ av fast kontakt ska anges med kod från kodverket Typ av fast kontakt, med text eller med båda. Koder från andra kodverk får inte användas. {(coding.exists() or text.exists()) and coding.all(system = 'https://fhir.inera.se/ig/careteam/CodeSystem/&lt;id&gt;')}</t>
+fast-kontakt-typ-kod-eller-text:Typ av fast kontakt ska anges med kod från kodverket Typ av fast kontakt, med text eller med båda. Koder från andra kodverk får inte användas. {(coding.exists() or text.exists()) and coding.all(system = 'https://terminologitjansten.inera.se/inera-kodverksforvaltning/kodverk/kv_typ_av_fast_kontakt')}</t>
   </si>
   <si>
     <t>Fast kontakt.typ</t>

</xml_diff>

<commit_message>
deploy: feature/careteam → branches/feature-careteam 221ffe2666ba767eff3ecb6efb5a3097368bd25f
</commit_message>
<xml_diff>
--- a/branches/feature-careteam/StructureDefinition-riv-care-manager-careteam.xlsx
+++ b/branches/feature-careteam/StructureDefinition-riv-care-manager-careteam.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-15T12:49:20+00:00</t>
+    <t>2026-10-15T13:32:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -237,7 +237,7 @@
     <t>Constraint(s)</t>
   </si>
   <si>
-    <t>Mapping: Mappning mellan informationsmodell och Fast kontakt</t>
+    <t>Mapping: Informationsmodell - Fast kontakt</t>
   </si>
   <si>
     <t>Mapping: FiveWs Pattern Mapping</t>
@@ -1924,7 +1924,7 @@
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="58.43359375" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="40.171875" customWidth="true" bestFit="true"/>
     <col min="38" max="38" width="31.65234375" customWidth="true" bestFit="true"/>
     <col min="39" max="39" width="39.890625" customWidth="true" bestFit="true"/>
     <col min="40" max="40" width="45.140625" customWidth="true" bestFit="true"/>

</xml_diff>